<commit_message>
Show three opening outcome classes for daily top two
</commit_message>
<xml_diff>
--- a/docs/stock_automl_runs/20261009_second_high_regression/daily_top2_review.xlsx
+++ b/docs/stock_automl_runs/20261009_second_high_regression/daily_top2_review.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="前二高开明细" sheetId="1" r:id="R8db36dc481db4925"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="逐日结果" sheetId="2" r:id="Rd744cc5314d3470d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="前二高开明细" sheetId="1" r:id="R6f09c13b26cf49a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="逐日结果" sheetId="2" r:id="Rd0bcfac560d241ff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -119,21 +119,23 @@
     <x:tableColumn id="7" name="14:40买价"/>
     <x:tableColumn id="8" name="十分钟最高开盘价"/>
     <x:tableColumn id="9" name="开盘涨幅"/>
-    <x:tableColumn id="10" name="高开&gt;1%?"/>
+    <x:tableColumn id="10" name="类别"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="OpenTop2Daily" displayName="OpenTop2Daily" ref="A4:F24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="6">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="OpenTop2Daily" displayName="OpenTop2Daily" ref="A4:H24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
     <x:tableColumn id="1" name="信号日"/>
     <x:tableColumn id="2" name="第一名"/>
     <x:tableColumn id="3" name="第一名开盘涨幅"/>
     <x:tableColumn id="4" name="第二名"/>
     <x:tableColumn id="5" name="第二名开盘涨幅"/>
-    <x:tableColumn id="6" name="高开只数"/>
+    <x:tableColumn id="6" name="达标"/>
+    <x:tableColumn id="7" name="中性"/>
+    <x:tableColumn id="8" name="严重错误"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -343,12 +345,12 @@
     <x:col min="7" max="7" width="19" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="19" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="19" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="13" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="15" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>每天前二：次日开盘十分钟是否高开</x:v>
+        <x:v>每天前二：次日开盘十分钟三档结果</x:v>
       </x:c>
       <x:c r="B1" s="6"/>
       <x:c r="C1" s="6"/>
@@ -362,7 +364,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="7" t="str">
-        <x:v>高开口径：09:31–09:40 十根精确 1 分钟 K 的最高开盘价，比信号日 14:40 买价高出超过 1%。</x:v>
+        <x:v>09:31–09:40 十根精确 1 分钟 K 的最高开盘价，相对信号日 14:40 买价：&gt;1% 达标，0–1% 中性，&lt;0% 严重错误。</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -403,7 +405,7 @@
         <x:v>开盘涨幅</x:v>
       </x:c>
       <x:c r="J4" s="9" t="str">
-        <x:v>高开&gt;1%?</x:v>
+        <x:v>类别</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -436,8 +438,8 @@
         <x:v>0.03256126216851296</x:v>
       </x:c>
       <x:c r="J5" s="10" t="str">
-        <x:f>IF(I5&gt;1%,"是","否")</x:f>
-        <x:v>是</x:v>
+        <x:f>IF(I5&gt;1%,"达标",IF(I5&lt;0,"严重错误","中性"))</x:f>
+        <x:v>达标</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -470,8 +472,8 @@
         <x:v>0.030160706201901366</x:v>
       </x:c>
       <x:c r="J6" s="10" t="str">
-        <x:f>IF(I6&gt;1%,"是","否")</x:f>
-        <x:v>是</x:v>
+        <x:f>IF(I6&gt;1%,"达标",IF(I6&lt;0,"严重错误","中性"))</x:f>
+        <x:v>达标</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -504,8 +506,8 @@
         <x:v>0.03835569315445464</x:v>
       </x:c>
       <x:c r="J7" s="10" t="str">
-        <x:f>IF(I7&gt;1%,"是","否")</x:f>
-        <x:v>是</x:v>
+        <x:f>IF(I7&gt;1%,"达标",IF(I7&lt;0,"严重错误","中性"))</x:f>
+        <x:v>达标</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -538,8 +540,8 @@
         <x:v>0.015331505736623008</x:v>
       </x:c>
       <x:c r="J8" s="10" t="str">
-        <x:f>IF(I8&gt;1%,"是","否")</x:f>
-        <x:v>是</x:v>
+        <x:f>IF(I8&gt;1%,"达标",IF(I8&lt;0,"严重错误","中性"))</x:f>
+        <x:v>达标</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -572,8 +574,8 @@
         <x:v>0.019625334522747506</x:v>
       </x:c>
       <x:c r="J9" s="10" t="str">
-        <x:f>IF(I9&gt;1%,"是","否")</x:f>
-        <x:v>是</x:v>
+        <x:f>IF(I9&gt;1%,"达标",IF(I9&lt;0,"严重错误","中性"))</x:f>
+        <x:v>达标</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -606,8 +608,8 @@
         <x:v>-0.0017452006980803736</x:v>
       </x:c>
       <x:c r="J10" s="10" t="str">
-        <x:f>IF(I10&gt;1%,"是","否")</x:f>
-        <x:v>否</x:v>
+        <x:f>IF(I10&gt;1%,"达标",IF(I10&lt;0,"严重错误","中性"))</x:f>
+        <x:v>严重错误</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -640,8 +642,8 @@
         <x:v>0.022264329701563224</x:v>
       </x:c>
       <x:c r="J11" s="10" t="str">
-        <x:f>IF(I11&gt;1%,"是","否")</x:f>
-        <x:v>是</x:v>
+        <x:f>IF(I11&gt;1%,"达标",IF(I11&lt;0,"严重错误","中性"))</x:f>
+        <x:v>达标</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -674,8 +676,8 @@
         <x:v>0.009110714993068036</x:v>
       </x:c>
       <x:c r="J12" s="10" t="str">
-        <x:f>IF(I12&gt;1%,"是","否")</x:f>
-        <x:v>否</x:v>
+        <x:f>IF(I12&gt;1%,"达标",IF(I12&lt;0,"严重错误","中性"))</x:f>
+        <x:v>中性</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -708,8 +710,8 @@
         <x:v>-0.029019346230820586</x:v>
       </x:c>
       <x:c r="J13" s="10" t="str">
-        <x:f>IF(I13&gt;1%,"是","否")</x:f>
-        <x:v>否</x:v>
+        <x:f>IF(I13&gt;1%,"达标",IF(I13&lt;0,"严重错误","中性"))</x:f>
+        <x:v>严重错误</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -742,8 +744,8 @@
         <x:v>0.007921998781230899</x:v>
       </x:c>
       <x:c r="J14" s="10" t="str">
-        <x:f>IF(I14&gt;1%,"是","否")</x:f>
-        <x:v>否</x:v>
+        <x:f>IF(I14&gt;1%,"达标",IF(I14&lt;0,"严重错误","中性"))</x:f>
+        <x:v>中性</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -776,8 +778,8 @@
         <x:v>-0.0099125364431486</x:v>
       </x:c>
       <x:c r="J15" s="10" t="str">
-        <x:f>IF(I15&gt;1%,"是","否")</x:f>
-        <x:v>否</x:v>
+        <x:f>IF(I15&gt;1%,"达标",IF(I15&lt;0,"严重错误","中性"))</x:f>
+        <x:v>严重错误</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -810,8 +812,8 @@
         <x:v>0.00872235325530668</x:v>
       </x:c>
       <x:c r="J16" s="10" t="str">
-        <x:f>IF(I16&gt;1%,"是","否")</x:f>
-        <x:v>否</x:v>
+        <x:f>IF(I16&gt;1%,"达标",IF(I16&lt;0,"严重错误","中性"))</x:f>
+        <x:v>中性</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -844,8 +846,8 @@
         <x:v>-0.016284987277353724</x:v>
       </x:c>
       <x:c r="J17" s="10" t="str">
-        <x:f>IF(I17&gt;1%,"是","否")</x:f>
-        <x:v>否</x:v>
+        <x:f>IF(I17&gt;1%,"达标",IF(I17&lt;0,"严重错误","中性"))</x:f>
+        <x:v>严重错误</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -878,8 +880,8 @@
         <x:v>-0.024436149189121403</x:v>
       </x:c>
       <x:c r="J18" s="10" t="str">
-        <x:f>IF(I18&gt;1%,"是","否")</x:f>
-        <x:v>否</x:v>
+        <x:f>IF(I18&gt;1%,"达标",IF(I18&lt;0,"严重错误","中性"))</x:f>
+        <x:v>严重错误</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -912,8 +914,8 @@
         <x:v>-0.021374045801526798</x:v>
       </x:c>
       <x:c r="J19" s="10" t="str">
-        <x:f>IF(I19&gt;1%,"是","否")</x:f>
-        <x:v>否</x:v>
+        <x:f>IF(I19&gt;1%,"达标",IF(I19&lt;0,"严重错误","中性"))</x:f>
+        <x:v>严重错误</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -946,8 +948,8 @@
         <x:v>0.025684931506849473</x:v>
       </x:c>
       <x:c r="J20" s="10" t="str">
-        <x:f>IF(I20&gt;1%,"是","否")</x:f>
-        <x:v>是</x:v>
+        <x:f>IF(I20&gt;1%,"达标",IF(I20&lt;0,"严重错误","中性"))</x:f>
+        <x:v>达标</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -980,8 +982,8 @@
         <x:v>0.02495974235104681</x:v>
       </x:c>
       <x:c r="J21" s="10" t="str">
-        <x:f>IF(I21&gt;1%,"是","否")</x:f>
-        <x:v>是</x:v>
+        <x:f>IF(I21&gt;1%,"达标",IF(I21&lt;0,"严重错误","中性"))</x:f>
+        <x:v>达标</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -1014,8 +1016,8 @@
         <x:v>-0.001890359168241984</x:v>
       </x:c>
       <x:c r="J22" s="10" t="str">
-        <x:f>IF(I22&gt;1%,"是","否")</x:f>
-        <x:v>否</x:v>
+        <x:f>IF(I22&gt;1%,"达标",IF(I22&lt;0,"严重错误","中性"))</x:f>
+        <x:v>严重错误</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -1048,8 +1050,8 @@
         <x:v>0.02315742596303738</x:v>
       </x:c>
       <x:c r="J23" s="10" t="str">
-        <x:f>IF(I23&gt;1%,"是","否")</x:f>
-        <x:v>是</x:v>
+        <x:f>IF(I23&gt;1%,"达标",IF(I23&lt;0,"严重错误","中性"))</x:f>
+        <x:v>达标</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1082,8 +1084,8 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J24" s="10" t="str">
-        <x:f>IF(I24&gt;1%,"是","否")</x:f>
-        <x:v>否</x:v>
+        <x:f>IF(I24&gt;1%,"达标",IF(I24&lt;0,"严重错误","中性"))</x:f>
+        <x:v>中性</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -1116,8 +1118,8 @@
         <x:v>0.11005792522380209</x:v>
       </x:c>
       <x:c r="J25" s="10" t="str">
-        <x:f>IF(I25&gt;1%,"是","否")</x:f>
-        <x:v>是</x:v>
+        <x:f>IF(I25&gt;1%,"达标",IF(I25&lt;0,"严重错误","中性"))</x:f>
+        <x:v>达标</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1150,8 +1152,8 @@
         <x:v>0.01721228484643955</x:v>
       </x:c>
       <x:c r="J26" s="10" t="str">
-        <x:f>IF(I26&gt;1%,"是","否")</x:f>
-        <x:v>是</x:v>
+        <x:f>IF(I26&gt;1%,"达标",IF(I26&lt;0,"严重错误","中性"))</x:f>
+        <x:v>达标</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -1184,8 +1186,8 @@
         <x:v>-0.0015503875968991832</x:v>
       </x:c>
       <x:c r="J27" s="10" t="str">
-        <x:f>IF(I27&gt;1%,"是","否")</x:f>
-        <x:v>否</x:v>
+        <x:f>IF(I27&gt;1%,"达标",IF(I27&lt;0,"严重错误","中性"))</x:f>
+        <x:v>严重错误</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -1218,8 +1220,8 @@
         <x:v>0.025983951089033175</x:v>
       </x:c>
       <x:c r="J28" s="10" t="str">
-        <x:f>IF(I28&gt;1%,"是","否")</x:f>
-        <x:v>是</x:v>
+        <x:f>IF(I28&gt;1%,"达标",IF(I28&lt;0,"严重错误","中性"))</x:f>
+        <x:v>达标</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -1252,8 +1254,8 @@
         <x:v>0.039981251464729306</x:v>
       </x:c>
       <x:c r="J29" s="10" t="str">
-        <x:f>IF(I29&gt;1%,"是","否")</x:f>
-        <x:v>是</x:v>
+        <x:f>IF(I29&gt;1%,"达标",IF(I29&lt;0,"严重错误","中性"))</x:f>
+        <x:v>达标</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -1286,8 +1288,8 @@
         <x:v>0.028353964536634413</x:v>
       </x:c>
       <x:c r="J30" s="10" t="str">
-        <x:f>IF(I30&gt;1%,"是","否")</x:f>
-        <x:v>是</x:v>
+        <x:f>IF(I30&gt;1%,"达标",IF(I30&lt;0,"严重错误","中性"))</x:f>
+        <x:v>达标</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -1320,8 +1322,8 @@
         <x:v>0.02139917695473259</x:v>
       </x:c>
       <x:c r="J31" s="10" t="str">
-        <x:f>IF(I31&gt;1%,"是","否")</x:f>
-        <x:v>是</x:v>
+        <x:f>IF(I31&gt;1%,"达标",IF(I31&lt;0,"严重错误","中性"))</x:f>
+        <x:v>达标</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -1354,8 +1356,8 @@
         <x:v>0.02244508118433619</x:v>
       </x:c>
       <x:c r="J32" s="10" t="str">
-        <x:f>IF(I32&gt;1%,"是","否")</x:f>
-        <x:v>是</x:v>
+        <x:f>IF(I32&gt;1%,"达标",IF(I32&lt;0,"严重错误","中性"))</x:f>
+        <x:v>达标</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -1388,8 +1390,8 @@
         <x:v>0.020068415051311295</x:v>
       </x:c>
       <x:c r="J33" s="10" t="str">
-        <x:f>IF(I33&gt;1%,"是","否")</x:f>
-        <x:v>是</x:v>
+        <x:f>IF(I33&gt;1%,"达标",IF(I33&lt;0,"严重错误","中性"))</x:f>
+        <x:v>达标</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -1422,8 +1424,8 @@
         <x:v>0.03240908907454498</x:v>
       </x:c>
       <x:c r="J34" s="10" t="str">
-        <x:f>IF(I34&gt;1%,"是","否")</x:f>
-        <x:v>是</x:v>
+        <x:f>IF(I34&gt;1%,"达标",IF(I34&lt;0,"严重错误","中性"))</x:f>
+        <x:v>达标</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -1456,8 +1458,8 @@
         <x:v>0.039170506912442615</x:v>
       </x:c>
       <x:c r="J35" s="10" t="str">
-        <x:f>IF(I35&gt;1%,"是","否")</x:f>
-        <x:v>是</x:v>
+        <x:f>IF(I35&gt;1%,"达标",IF(I35&lt;0,"严重错误","中性"))</x:f>
+        <x:v>达标</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -1490,8 +1492,8 @@
         <x:v>-0.0019762845849801147</x:v>
       </x:c>
       <x:c r="J36" s="10" t="str">
-        <x:f>IF(I36&gt;1%,"是","否")</x:f>
-        <x:v>否</x:v>
+        <x:f>IF(I36&gt;1%,"达标",IF(I36&lt;0,"严重错误","中性"))</x:f>
+        <x:v>严重错误</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -1524,8 +1526,8 @@
         <x:v>0.09357030841610059</x:v>
       </x:c>
       <x:c r="J37" s="10" t="str">
-        <x:f>IF(I37&gt;1%,"是","否")</x:f>
-        <x:v>是</x:v>
+        <x:f>IF(I37&gt;1%,"达标",IF(I37&lt;0,"严重错误","中性"))</x:f>
+        <x:v>达标</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -1558,8 +1560,8 @@
         <x:v>0.009236067626800182</x:v>
       </x:c>
       <x:c r="J38" s="10" t="str">
-        <x:f>IF(I38&gt;1%,"是","否")</x:f>
-        <x:v>否</x:v>
+        <x:f>IF(I38&gt;1%,"达标",IF(I38&lt;0,"严重错误","中性"))</x:f>
+        <x:v>中性</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -1592,8 +1594,8 @@
         <x:v>0.03886255924170623</x:v>
       </x:c>
       <x:c r="J39" s="10" t="str">
-        <x:f>IF(I39&gt;1%,"是","否")</x:f>
-        <x:v>是</x:v>
+        <x:f>IF(I39&gt;1%,"达标",IF(I39&lt;0,"严重错误","中性"))</x:f>
+        <x:v>达标</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -1626,8 +1628,8 @@
         <x:v>-0.031061929722384085</x:v>
       </x:c>
       <x:c r="J40" s="10" t="str">
-        <x:f>IF(I40&gt;1%,"是","否")</x:f>
-        <x:v>否</x:v>
+        <x:f>IF(I40&gt;1%,"达标",IF(I40&lt;0,"严重错误","中性"))</x:f>
+        <x:v>严重错误</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -1660,8 +1662,8 @@
         <x:v>-0.001151189562547894</x:v>
       </x:c>
       <x:c r="J41" s="10" t="str">
-        <x:f>IF(I41&gt;1%,"是","否")</x:f>
-        <x:v>否</x:v>
+        <x:f>IF(I41&gt;1%,"达标",IF(I41&lt;0,"严重错误","中性"))</x:f>
+        <x:v>严重错误</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -1694,8 +1696,8 @@
         <x:v>0.03060514722930674</x:v>
       </x:c>
       <x:c r="J42" s="10" t="str">
-        <x:f>IF(I42&gt;1%,"是","否")</x:f>
-        <x:v>是</x:v>
+        <x:f>IF(I42&gt;1%,"达标",IF(I42&lt;0,"严重错误","中性"))</x:f>
+        <x:v>达标</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -1728,8 +1730,8 @@
         <x:v>-0.007912957467853587</x:v>
       </x:c>
       <x:c r="J43" s="10" t="str">
-        <x:f>IF(I43&gt;1%,"是","否")</x:f>
-        <x:v>否</x:v>
+        <x:f>IF(I43&gt;1%,"达标",IF(I43&lt;0,"严重错误","中性"))</x:f>
+        <x:v>严重错误</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -1762,8 +1764,8 @@
         <x:v>0.06632653061224492</x:v>
       </x:c>
       <x:c r="J44" s="10" t="str">
-        <x:f>IF(I44&gt;1%,"是","否")</x:f>
-        <x:v>是</x:v>
+        <x:f>IF(I44&gt;1%,"达标",IF(I44&lt;0,"严重错误","中性"))</x:f>
+        <x:v>达标</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1773,7 +1775,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80a601699f704ef0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ec3a172480c44ca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1787,28 +1789,34 @@
     <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="17" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>每天两只高开了几只</x:v>
+        <x:v>每天前二的达标 / 中性 / 严重错误</x:v>
       </x:c>
       <x:c r="B1" s="6"/>
       <x:c r="C1" s="6"/>
       <x:c r="D1" s="6"/>
       <x:c r="E1" s="6"/>
       <x:c r="F1" s="6"/>
+      <x:c r="G1" s="6"/>
+      <x:c r="H1" s="6"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="7" t="str">
-        <x:v>是 = 十分钟最高开盘价相对 14:40 买价涨超 1%；每个测试日固定取模型前二。</x:v>
+        <x:v>开盘十分钟最高开盘价相对 14:40 买价：&gt;1% 达标，0–1% 中性，&lt;0% 严重错误。</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
       <x:c r="D2" s="7"/>
       <x:c r="E2" s="7"/>
       <x:c r="F2" s="7"/>
+      <x:c r="G2" s="7"/>
+      <x:c r="H2" s="7"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="9" t="str">
@@ -1827,7 +1835,13 @@
         <x:v>第二名开盘涨幅</x:v>
       </x:c>
       <x:c r="F4" s="9" t="str">
-        <x:v>高开只数</x:v>
+        <x:v>达标</x:v>
+      </x:c>
+      <x:c r="G4" s="9" t="str">
+        <x:v>中性</x:v>
+      </x:c>
+      <x:c r="H4" s="9" t="str">
+        <x:v>严重错误</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1852,8 +1866,16 @@
         <x:v>0.030160706201901366</x:v>
       </x:c>
       <x:c r="F5" s="10" t="n">
-        <x:f>COUNTIF('前二高开明细'!J5:J6,"是")</x:f>
-        <x:v>2</x:v>
+        <x:f>COUNTIF('前二高开明细'!J5:J6,"达标")</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G5" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J5:J6,"中性")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H5" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J5:J6,"严重错误")</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1878,8 +1900,16 @@
         <x:v>0.015331505736623008</x:v>
       </x:c>
       <x:c r="F6" s="10" t="n">
-        <x:f>COUNTIF('前二高开明细'!J7:J8,"是")</x:f>
-        <x:v>2</x:v>
+        <x:f>COUNTIF('前二高开明细'!J7:J8,"达标")</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G6" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J7:J8,"中性")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H6" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J7:J8,"严重错误")</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1904,7 +1934,15 @@
         <x:v>-0.0017452006980803736</x:v>
       </x:c>
       <x:c r="F7" s="10" t="n">
-        <x:f>COUNTIF('前二高开明细'!J9:J10,"是")</x:f>
+        <x:f>COUNTIF('前二高开明细'!J9:J10,"达标")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G7" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J9:J10,"中性")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H7" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J9:J10,"严重错误")</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -1930,8 +1968,16 @@
         <x:v>0.009110714993068036</x:v>
       </x:c>
       <x:c r="F8" s="10" t="n">
-        <x:f>COUNTIF('前二高开明细'!J11:J12,"是")</x:f>
-        <x:v>1</x:v>
+        <x:f>COUNTIF('前二高开明细'!J11:J12,"达标")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G8" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J11:J12,"中性")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H8" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J11:J12,"严重错误")</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1956,8 +2002,16 @@
         <x:v>0.007921998781230899</x:v>
       </x:c>
       <x:c r="F9" s="10" t="n">
-        <x:f>COUNTIF('前二高开明细'!J13:J14,"是")</x:f>
-        <x:v>0</x:v>
+        <x:f>COUNTIF('前二高开明细'!J13:J14,"达标")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G9" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J13:J14,"中性")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H9" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J13:J14,"严重错误")</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1982,8 +2036,16 @@
         <x:v>0.00872235325530668</x:v>
       </x:c>
       <x:c r="F10" s="10" t="n">
-        <x:f>COUNTIF('前二高开明细'!J15:J16,"是")</x:f>
-        <x:v>0</x:v>
+        <x:f>COUNTIF('前二高开明细'!J15:J16,"达标")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G10" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J15:J16,"中性")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H10" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J15:J16,"严重错误")</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2008,8 +2070,16 @@
         <x:v>-0.024436149189121403</x:v>
       </x:c>
       <x:c r="F11" s="10" t="n">
-        <x:f>COUNTIF('前二高开明细'!J17:J18,"是")</x:f>
-        <x:v>0</x:v>
+        <x:f>COUNTIF('前二高开明细'!J17:J18,"达标")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G11" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J17:J18,"中性")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H11" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J17:J18,"严重错误")</x:f>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -2034,7 +2104,15 @@
         <x:v>0.025684931506849473</x:v>
       </x:c>
       <x:c r="F12" s="10" t="n">
-        <x:f>COUNTIF('前二高开明细'!J19:J20,"是")</x:f>
+        <x:f>COUNTIF('前二高开明细'!J19:J20,"达标")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G12" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J19:J20,"中性")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H12" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J19:J20,"严重错误")</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -2060,7 +2138,15 @@
         <x:v>-0.001890359168241984</x:v>
       </x:c>
       <x:c r="F13" s="10" t="n">
-        <x:f>COUNTIF('前二高开明细'!J21:J22,"是")</x:f>
+        <x:f>COUNTIF('前二高开明细'!J21:J22,"达标")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G13" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J21:J22,"中性")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H13" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J21:J22,"严重错误")</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -2086,8 +2172,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F14" s="10" t="n">
-        <x:f>COUNTIF('前二高开明细'!J23:J24,"是")</x:f>
-        <x:v>1</x:v>
+        <x:f>COUNTIF('前二高开明细'!J23:J24,"达标")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G14" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J23:J24,"中性")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H14" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J23:J24,"严重错误")</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2112,8 +2206,16 @@
         <x:v>0.01721228484643955</x:v>
       </x:c>
       <x:c r="F15" s="10" t="n">
-        <x:f>COUNTIF('前二高开明细'!J25:J26,"是")</x:f>
-        <x:v>2</x:v>
+        <x:f>COUNTIF('前二高开明细'!J25:J26,"达标")</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G15" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J25:J26,"中性")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H15" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J25:J26,"严重错误")</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -2138,7 +2240,15 @@
         <x:v>0.025983951089033175</x:v>
       </x:c>
       <x:c r="F16" s="10" t="n">
-        <x:f>COUNTIF('前二高开明细'!J27:J28,"是")</x:f>
+        <x:f>COUNTIF('前二高开明细'!J27:J28,"达标")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G16" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J27:J28,"中性")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H16" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J27:J28,"严重错误")</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -2164,8 +2274,16 @@
         <x:v>0.028353964536634413</x:v>
       </x:c>
       <x:c r="F17" s="10" t="n">
-        <x:f>COUNTIF('前二高开明细'!J29:J30,"是")</x:f>
-        <x:v>2</x:v>
+        <x:f>COUNTIF('前二高开明细'!J29:J30,"达标")</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G17" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J29:J30,"中性")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H17" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J29:J30,"严重错误")</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2190,8 +2308,16 @@
         <x:v>0.02244508118433619</x:v>
       </x:c>
       <x:c r="F18" s="10" t="n">
-        <x:f>COUNTIF('前二高开明细'!J31:J32,"是")</x:f>
-        <x:v>2</x:v>
+        <x:f>COUNTIF('前二高开明细'!J31:J32,"达标")</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G18" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J31:J32,"中性")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H18" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J31:J32,"严重错误")</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -2216,8 +2342,16 @@
         <x:v>0.03240908907454498</x:v>
       </x:c>
       <x:c r="F19" s="10" t="n">
-        <x:f>COUNTIF('前二高开明细'!J33:J34,"是")</x:f>
-        <x:v>2</x:v>
+        <x:f>COUNTIF('前二高开明细'!J33:J34,"达标")</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G19" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J33:J34,"中性")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H19" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J33:J34,"严重错误")</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -2242,7 +2376,15 @@
         <x:v>-0.0019762845849801147</x:v>
       </x:c>
       <x:c r="F20" s="10" t="n">
-        <x:f>COUNTIF('前二高开明细'!J35:J36,"是")</x:f>
+        <x:f>COUNTIF('前二高开明细'!J35:J36,"达标")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G20" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J35:J36,"中性")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H20" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J35:J36,"严重错误")</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -2268,8 +2410,16 @@
         <x:v>0.009236067626800182</x:v>
       </x:c>
       <x:c r="F21" s="10" t="n">
-        <x:f>COUNTIF('前二高开明细'!J37:J38,"是")</x:f>
-        <x:v>1</x:v>
+        <x:f>COUNTIF('前二高开明细'!J37:J38,"达标")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G21" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J37:J38,"中性")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H21" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J37:J38,"严重错误")</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -2294,7 +2444,15 @@
         <x:v>-0.031061929722384085</x:v>
       </x:c>
       <x:c r="F22" s="10" t="n">
-        <x:f>COUNTIF('前二高开明细'!J39:J40,"是")</x:f>
+        <x:f>COUNTIF('前二高开明细'!J39:J40,"达标")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G22" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J39:J40,"中性")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H22" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J39:J40,"严重错误")</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -2320,7 +2478,15 @@
         <x:v>0.03060514722930674</x:v>
       </x:c>
       <x:c r="F23" s="10" t="n">
-        <x:f>COUNTIF('前二高开明细'!J41:J42,"是")</x:f>
+        <x:f>COUNTIF('前二高开明细'!J41:J42,"达标")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G23" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J41:J42,"中性")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H23" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J41:J42,"严重错误")</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -2346,7 +2512,15 @@
         <x:v>0.06632653061224492</x:v>
       </x:c>
       <x:c r="F24" s="10" t="n">
-        <x:f>COUNTIF('前二高开明细'!J43:J44,"是")</x:f>
+        <x:f>COUNTIF('前二高开明细'!J43:J44,"达标")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G24" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J43:J44,"中性")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H24" s="10" t="n">
+        <x:f>COUNTIF('前二高开明细'!J43:J44,"严重错误")</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -2357,6 +2531,8 @@
       <x:c r="D25" s="10"/>
       <x:c r="E25" s="10"/>
       <x:c r="F25" s="10"/>
+      <x:c r="G25" s="10"/>
+      <x:c r="H25" s="10"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="10"/>
@@ -2365,6 +2541,8 @@
       <x:c r="D26" s="10"/>
       <x:c r="E26" s="10"/>
       <x:c r="F26" s="10"/>
+      <x:c r="G26" s="10"/>
+      <x:c r="H26" s="10"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="16" t="str">
@@ -2380,15 +2558,23 @@
         <x:f>SUM(F5:F24)</x:f>
         <x:v>23</x:v>
       </x:c>
+      <x:c r="G27" s="16" t="n">
+        <x:f>SUM(G5:G24)</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H27" s="16" t="n">
+        <x:f>SUM(H5:H24)</x:f>
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:F1"/>
-    <x:mergeCell ref="A2:F2"/>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6217479244fc4cf7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b364a1aeed24052"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>